<commit_message>
Enhance Excel and Word file handling in generate.py with improved error messages and data structure. Introduce SheetData class for better organization of sheet data and validate input sheets for required columns and data presence.
</commit_message>
<xml_diff>
--- a/input/作品情報フォーム.xlsx
+++ b/input/作品情報フォーム.xlsx
@@ -5,19 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ka5ry\Documents\work\kushodo_brochure_gen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ka5ry\Documents\work\kushodo_brochure_gen\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79139C28-460F-4EC8-B9EA-1A09B35F1706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB7F691-BC64-457A-9500-AC5C325E08F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="個人" sheetId="2" r:id="rId1"/>
     <sheet name="合作" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -899,22 +898,6 @@
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1059,31 +1042,47 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="4">
     <tableStyle name="第二回個人-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="12"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="secondRowStripe" dxfId="13"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="15"/>
+      <tableStyleElement type="headerRow" dxfId="14"/>
+      <tableStyleElement type="firstRowStripe" dxfId="13"/>
+      <tableStyleElement type="secondRowStripe" dxfId="12"/>
     </tableStyle>
     <tableStyle name="第二回合作-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="8"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
-      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
+      <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
     <tableStyle name="フォームの回答 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="フォームの回答 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>

</xml_diff>

<commit_message>
Update main.tsx to consolidate header text for the brochure generation page and modify an Excel file in the input directory.
</commit_message>
<xml_diff>
--- a/input/作品情報フォーム.xlsx
+++ b/input/作品情報フォーム.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ka5ry\Documents\work\kushodo_brochure_gen\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB7F691-BC64-457A-9500-AC5C325E08F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9EB1F6F-2C5B-453C-A8A9-4F414BD7866F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="17280" windowHeight="10665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="個人" sheetId="2" r:id="rId1"/>

</xml_diff>